<commit_message>
Continue manual edits on 05.4b_edited3
</commit_message>
<xml_diff>
--- a/data/data-wrangling-intermediate/05.4b_edited3_LDC_multiple-same-DateVisted.xlsx
+++ b/data/data-wrangling-intermediate/05.4b_edited3_LDC_multiple-same-DateVisted.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eltnmsu-my.sharepoint.com/personal/lossanna_nmsu_edu/Documents/Documents/04_LDC-LTDL/LDC-LTDL/data/data-wrangling-intermediate/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="271" documentId="8_{A0E79672-A511-4ABE-8E84-8B3C26D93CC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{63F485D5-5634-4118-B53E-ABABC21FA930}"/>
+  <xr:revisionPtr revIDLastSave="368" documentId="8_{A0E79672-A511-4ABE-8E84-8B3C26D93CC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5F0A082B-FCF7-4F01-A3A8-7504C1A51E3E}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{AD8A9A48-ECC0-46BC-9F8C-90AF05074D89}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2654" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2668" uniqueCount="211">
   <si>
     <t>ProjKey</t>
   </si>
@@ -620,9 +620,6 @@
     <t>identical data?</t>
   </si>
   <si>
-    <t>flux &amp; LT missing in second, EcoSiteID differs</t>
-  </si>
-  <si>
     <t>height differs</t>
   </si>
   <si>
@@ -654,13 +651,16 @@
   </si>
   <si>
     <t>drop</t>
+  </si>
+  <si>
+    <t>flux &amp; LT missing in second, EcoSiteID unknown in first</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -791,6 +791,19 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0" tint="-0.499984740745262"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1172,7 +1185,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
@@ -1187,16 +1200,20 @@
     <xf numFmtId="0" fontId="0" fillId="33" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="14" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="14" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="18" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="18" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="18" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="14" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="14" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1267,8 +1284,8 @@
     <xdr:to>
       <xdr:col>9</xdr:col>
       <xdr:colOff>563880</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1284,7 +1301,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="998220" y="662940"/>
-          <a:ext cx="5052060" cy="1021080"/>
+          <a:ext cx="5052060" cy="1226820"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1361,7 +1378,32 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>Red text = drop row</a:t>
+            <a:t>Gray text = drop row</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="en-US" sz="1100" baseline="0">
+            <a:solidFill>
+              <a:schemeClr val="dk1"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Red text = replaced for row to keep ("UNKNOWN" replaced with the EcoSiteID from the other row)</a:t>
           </a:r>
           <a:endParaRPr lang="en-US" sz="1100"/>
         </a:p>
@@ -1735,7 +1777,7 @@
         <v>197</v>
       </c>
       <c r="E1" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F1" t="s">
         <v>2</v>
@@ -1989,7 +2031,7 @@
         <v>109</v>
       </c>
       <c r="D2" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F2" s="1">
         <v>41723</v>
@@ -2243,7 +2285,7 @@
         <v>111</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F3" s="3">
         <v>41723</v>
@@ -2497,7 +2539,7 @@
         <v>106</v>
       </c>
       <c r="D4" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F4" s="1">
         <v>41723</v>
@@ -2751,7 +2793,7 @@
         <v>108</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F5" s="3">
         <v>41723</v>
@@ -3005,7 +3047,7 @@
         <v>96</v>
       </c>
       <c r="D6" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F6" s="1">
         <v>41723</v>
@@ -3510,7 +3552,7 @@
         <v>151</v>
       </c>
       <c r="D8" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="F8" s="1">
         <v>43644</v>
@@ -4768,7 +4810,7 @@
         <v>84</v>
       </c>
       <c r="D13" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="F13" s="1">
         <v>44722</v>
@@ -5296,28 +5338,28 @@
       <c r="M15" s="9">
         <v>-114</v>
       </c>
-      <c r="N15" s="2">
+      <c r="N15" s="5">
         <v>2</v>
       </c>
-      <c r="O15" s="2">
+      <c r="O15" s="5">
         <v>10</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="5">
         <v>31</v>
       </c>
-      <c r="Q15" s="2">
+      <c r="Q15" s="5">
         <v>38</v>
       </c>
-      <c r="R15" s="2">
+      <c r="R15" s="5">
         <v>38</v>
       </c>
-      <c r="S15" s="2">
+      <c r="S15" s="5">
         <v>70</v>
       </c>
       <c r="T15" s="2">
         <v>30</v>
       </c>
-      <c r="U15" s="2">
+      <c r="U15" s="5">
         <v>50</v>
       </c>
       <c r="V15" s="2">
@@ -5326,7 +5368,7 @@
       <c r="W15" s="2">
         <v>0</v>
       </c>
-      <c r="X15" s="2">
+      <c r="X15" s="5">
         <v>3</v>
       </c>
       <c r="Y15" s="2">
@@ -5335,7 +5377,7 @@
       <c r="Z15" s="2">
         <v>0</v>
       </c>
-      <c r="AA15" s="2">
+      <c r="AA15" s="5">
         <v>0</v>
       </c>
       <c r="AB15" s="2">
@@ -5347,7 +5389,7 @@
       <c r="AD15" s="2">
         <v>0</v>
       </c>
-      <c r="AE15" s="2">
+      <c r="AE15" s="5">
         <v>2</v>
       </c>
       <c r="AF15" s="2">
@@ -5524,7 +5566,7 @@
         <v>192</v>
       </c>
       <c r="D16" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F16" s="1">
         <v>45127</v>
@@ -6280,7 +6322,7 @@
         <v>188</v>
       </c>
       <c r="D19" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F19" s="1">
         <v>43304</v>
@@ -6784,11 +6826,17 @@
       <c r="C21" t="s">
         <v>159</v>
       </c>
+      <c r="D21" t="s">
+        <v>210</v>
+      </c>
+      <c r="E21" t="s">
+        <v>208</v>
+      </c>
       <c r="F21" s="1">
         <v>43271</v>
       </c>
-      <c r="G21" t="s">
-        <v>97</v>
+      <c r="G21" s="24" t="s">
+        <v>130</v>
       </c>
       <c r="H21" t="s">
         <v>122</v>
@@ -7000,279 +7048,282 @@
       <c r="BY21" s="12">
         <v>45670</v>
       </c>
-      <c r="BZ21">
-        <v>0</v>
-      </c>
-      <c r="CA21">
-        <v>0</v>
-      </c>
-      <c r="CB21">
-        <v>0</v>
-      </c>
-      <c r="CC21">
-        <v>0</v>
-      </c>
-      <c r="CD21">
+      <c r="BZ21" s="4">
+        <v>0</v>
+      </c>
+      <c r="CA21" s="4">
+        <v>0</v>
+      </c>
+      <c r="CB21" s="4">
+        <v>0</v>
+      </c>
+      <c r="CC21" s="4">
+        <v>0</v>
+      </c>
+      <c r="CD21" s="4">
         <v>307</v>
       </c>
-      <c r="CE21">
+      <c r="CE21" s="4">
         <v>9</v>
       </c>
-      <c r="CF21">
-        <v>0</v>
-      </c>
-      <c r="CG21">
+      <c r="CF21" s="4">
+        <v>0</v>
+      </c>
+      <c r="CG21" s="4">
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:85" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="2">
+    <row r="22" spans="1:85" s="14" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="14">
         <v>48807</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="14" t="s">
         <v>95</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C22" s="14" t="s">
         <v>160</v>
       </c>
-      <c r="F22" s="3">
+      <c r="E22" s="14" t="s">
+        <v>209</v>
+      </c>
+      <c r="F22" s="15">
         <v>43271</v>
       </c>
-      <c r="G22" s="2" t="s">
+      <c r="G22" s="16" t="s">
         <v>130</v>
       </c>
-      <c r="H22" s="2" t="s">
+      <c r="H22" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="I22" s="2" t="s">
+      <c r="I22" s="14" t="s">
         <v>123</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="14">
         <v>13075</v>
       </c>
-      <c r="K22" s="2">
+      <c r="K22" s="14">
         <v>2</v>
       </c>
-      <c r="L22" s="2">
+      <c r="L22" s="14">
         <v>43.560200000000002</v>
       </c>
-      <c r="M22" s="9">
+      <c r="M22" s="17">
         <v>-106.36747</v>
       </c>
-      <c r="N22" s="2">
+      <c r="N22" s="14">
         <v>6.6666666666666696</v>
       </c>
-      <c r="O22" s="2">
+      <c r="O22" s="14">
         <v>8</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="14">
         <v>63.3333333333333</v>
       </c>
-      <c r="Q22" s="2">
+      <c r="Q22" s="14">
         <v>10.6666666666667</v>
       </c>
-      <c r="R22" s="2">
+      <c r="R22" s="14">
         <v>65.3333333333333</v>
       </c>
-      <c r="S22" s="2">
+      <c r="S22" s="14">
         <v>86</v>
       </c>
-      <c r="T22" s="2">
+      <c r="T22" s="14">
         <v>3.3333333333333299</v>
       </c>
-      <c r="U22" s="2">
+      <c r="U22" s="14">
         <v>62</v>
       </c>
-      <c r="V22" s="2">
+      <c r="V22" s="14">
         <v>11.3333333333333</v>
       </c>
-      <c r="W22" s="2">
-        <v>0</v>
-      </c>
-      <c r="X22" s="2">
-        <v>0</v>
-      </c>
-      <c r="Y22" s="2">
-        <v>0</v>
-      </c>
-      <c r="Z22" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA22" s="2">
+      <c r="W22" s="14">
+        <v>0</v>
+      </c>
+      <c r="X22" s="14">
+        <v>0</v>
+      </c>
+      <c r="Y22" s="14">
+        <v>0</v>
+      </c>
+      <c r="Z22" s="14">
+        <v>0</v>
+      </c>
+      <c r="AA22" s="14">
         <v>4.6666666666666696</v>
       </c>
-      <c r="AB22" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC22" s="2">
-        <v>0</v>
-      </c>
-      <c r="AD22" s="2">
-        <v>0</v>
-      </c>
-      <c r="AE22" s="2">
+      <c r="AB22" s="14">
+        <v>0</v>
+      </c>
+      <c r="AC22" s="14">
+        <v>0</v>
+      </c>
+      <c r="AD22" s="14">
+        <v>0</v>
+      </c>
+      <c r="AE22" s="14">
         <v>4.6666666666666696</v>
       </c>
-      <c r="AF22" s="2">
-        <v>0</v>
-      </c>
-      <c r="AG22" s="2">
-        <v>0</v>
-      </c>
-      <c r="AH22" s="9">
-        <v>0</v>
-      </c>
-      <c r="AI22" s="2">
+      <c r="AF22" s="14">
+        <v>0</v>
+      </c>
+      <c r="AG22" s="14">
+        <v>0</v>
+      </c>
+      <c r="AH22" s="17">
+        <v>0</v>
+      </c>
+      <c r="AI22" s="14">
         <v>1.88</v>
       </c>
-      <c r="AJ22" s="2">
-        <v>0</v>
-      </c>
-      <c r="AK22" s="2">
-        <v>0</v>
-      </c>
-      <c r="AL22" s="2">
-        <v>0</v>
-      </c>
-      <c r="AM22" s="9">
+      <c r="AJ22" s="14">
+        <v>0</v>
+      </c>
+      <c r="AK22" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL22" s="14">
+        <v>0</v>
+      </c>
+      <c r="AM22" s="17">
         <v>1.88</v>
       </c>
-      <c r="AN22" s="2">
+      <c r="AN22" s="14">
         <v>27</v>
       </c>
-      <c r="AO22" s="2">
+      <c r="AO22" s="14">
         <v>32.344827586206897</v>
       </c>
-      <c r="AP22" s="2">
+      <c r="AP22" s="14">
         <v>32.1666666666667</v>
       </c>
-      <c r="AQ22" s="2">
+      <c r="AQ22" s="14">
         <v>27</v>
       </c>
-      <c r="AR22" s="2">
+      <c r="AR22" s="14">
         <v>33.045454545454497</v>
       </c>
-      <c r="AS22" s="2">
+      <c r="AS22" s="14">
         <v>33.3333333333333</v>
       </c>
-      <c r="AT22" s="9">
+      <c r="AT22" s="17">
         <v>36.25</v>
       </c>
-      <c r="AU22" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="AV22" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="AW22" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="AX22" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="AY22" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="AZ22" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BA22" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BB22" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BC22" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BD22" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BE22" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BF22" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BG22" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BH22" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BI22" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BJ22" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BK22" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BL22" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BM22" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BN22" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BO22" s="2">
+      <c r="AU22" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="AV22" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="AW22" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="AX22" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="AY22" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="AZ22" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BA22" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BB22" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BC22" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BD22" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BE22" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BF22" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BG22" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BH22" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BI22" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BJ22" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BK22" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BL22" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BM22" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BN22" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BO22" s="14">
         <v>4.7777777777777803</v>
       </c>
-      <c r="BP22" s="2">
+      <c r="BP22" s="14">
         <v>4.9230769230769198</v>
       </c>
-      <c r="BQ22" s="2">
+      <c r="BQ22" s="14">
         <v>4.4000000000000004</v>
       </c>
-      <c r="BR22" s="2" t="s">
+      <c r="BR22" s="14" t="s">
         <v>124</v>
       </c>
-      <c r="BS22" s="2" t="s">
+      <c r="BS22" s="14" t="s">
         <v>125</v>
       </c>
-      <c r="BT22" s="2" t="s">
+      <c r="BT22" s="14" t="s">
         <v>126</v>
       </c>
-      <c r="BU22" s="2" t="s">
+      <c r="BU22" s="14" t="s">
         <v>127</v>
       </c>
-      <c r="BV22" s="2" t="s">
+      <c r="BV22" s="14" t="s">
         <v>118</v>
       </c>
-      <c r="BW22" s="2" t="s">
+      <c r="BW22" s="14" t="s">
         <v>92</v>
       </c>
-      <c r="BX22" s="2" t="s">
+      <c r="BX22" s="14" t="s">
         <v>104</v>
       </c>
-      <c r="BY22" s="13">
+      <c r="BY22" s="18">
         <v>45670</v>
       </c>
-      <c r="BZ22" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="CA22" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="CB22" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="CC22" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="CD22" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="CE22" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="CF22" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="CG22" s="2" t="s">
+      <c r="BZ22" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="CA22" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="CB22" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="CC22" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="CD22" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="CE22" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="CF22" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="CG22" s="16" t="s">
         <v>85</v>
       </c>
     </row>
@@ -7289,6 +7340,9 @@
       <c r="D23" t="s">
         <v>198</v>
       </c>
+      <c r="E23" t="s">
+        <v>208</v>
+      </c>
       <c r="F23" s="1">
         <v>43248</v>
       </c>
@@ -7530,254 +7584,257 @@
         <v>85</v>
       </c>
     </row>
-    <row r="24" spans="1:85" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="2">
+    <row r="24" spans="1:85" s="14" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="14">
         <v>48995</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="14" t="s">
         <v>95</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C24" s="14" t="s">
         <v>128</v>
       </c>
-      <c r="F24" s="3">
+      <c r="E24" s="14" t="s">
+        <v>209</v>
+      </c>
+      <c r="F24" s="15">
         <v>43248</v>
       </c>
-      <c r="G24" s="2" t="s">
+      <c r="G24" s="14" t="s">
         <v>121</v>
       </c>
-      <c r="H24" s="2" t="s">
+      <c r="H24" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="I24" s="2" t="s">
+      <c r="I24" s="14" t="s">
         <v>123</v>
       </c>
-      <c r="J24" s="2">
+      <c r="J24" s="14">
         <v>12207</v>
       </c>
-      <c r="K24" s="2">
+      <c r="K24" s="14">
         <v>2</v>
       </c>
-      <c r="L24" s="2">
+      <c r="L24" s="14">
         <v>43.601757999999997</v>
       </c>
-      <c r="M24" s="9">
+      <c r="M24" s="17">
         <v>-106.67084199999999</v>
       </c>
-      <c r="N24" s="2">
+      <c r="N24" s="14">
         <v>3.3333333333333299</v>
       </c>
-      <c r="O24" s="2">
+      <c r="O24" s="14">
         <v>6.6666666666666696</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="14">
         <v>62</v>
       </c>
-      <c r="Q24" s="2">
+      <c r="Q24" s="14">
         <v>7.3333333333333304</v>
       </c>
-      <c r="R24" s="2">
+      <c r="R24" s="14">
         <v>66.6666666666667</v>
       </c>
-      <c r="S24" s="2">
+      <c r="S24" s="14">
         <v>72.6666666666667</v>
       </c>
-      <c r="T24" s="2">
+      <c r="T24" s="14">
         <v>0.66666666666666696</v>
       </c>
-      <c r="U24" s="2">
+      <c r="U24" s="14">
         <v>28</v>
       </c>
-      <c r="V24" s="2">
+      <c r="V24" s="14">
         <v>14</v>
       </c>
-      <c r="W24" s="2">
-        <v>0</v>
-      </c>
-      <c r="X24" s="2">
-        <v>0</v>
-      </c>
-      <c r="Y24" s="2">
+      <c r="W24" s="14">
+        <v>0</v>
+      </c>
+      <c r="X24" s="14">
+        <v>0</v>
+      </c>
+      <c r="Y24" s="14">
         <v>0.66666666666666696</v>
       </c>
-      <c r="Z24" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA24" s="2">
+      <c r="Z24" s="14">
+        <v>0</v>
+      </c>
+      <c r="AA24" s="14">
         <v>10.6666666666667</v>
       </c>
-      <c r="AB24" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC24" s="2">
+      <c r="AB24" s="14">
+        <v>0</v>
+      </c>
+      <c r="AC24" s="14">
         <v>4.6666666666666696</v>
       </c>
-      <c r="AD24" s="2">
-        <v>0</v>
-      </c>
-      <c r="AE24" s="2">
+      <c r="AD24" s="14">
+        <v>0</v>
+      </c>
+      <c r="AE24" s="14">
         <v>11.3333333333333</v>
       </c>
-      <c r="AF24" s="2">
-        <v>0</v>
-      </c>
-      <c r="AG24" s="2">
-        <v>0</v>
-      </c>
-      <c r="AH24" s="9">
+      <c r="AF24" s="14">
+        <v>0</v>
+      </c>
+      <c r="AG24" s="14">
+        <v>0</v>
+      </c>
+      <c r="AH24" s="17">
         <v>0.66666666666666696</v>
       </c>
-      <c r="AI24" s="2">
+      <c r="AI24" s="14">
         <v>1.33</v>
       </c>
-      <c r="AJ24" s="2">
-        <v>0</v>
-      </c>
-      <c r="AK24" s="2">
-        <v>0</v>
-      </c>
-      <c r="AL24" s="2">
-        <v>0</v>
-      </c>
-      <c r="AM24" s="9">
+      <c r="AJ24" s="14">
+        <v>0</v>
+      </c>
+      <c r="AK24" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL24" s="14">
+        <v>0</v>
+      </c>
+      <c r="AM24" s="17">
         <v>1.33</v>
       </c>
-      <c r="AN24" s="2">
+      <c r="AN24" s="14">
         <v>13</v>
       </c>
-      <c r="AO24" s="2">
+      <c r="AO24" s="14">
         <v>32.517241379310299</v>
       </c>
-      <c r="AP24" s="2">
+      <c r="AP24" s="14">
         <v>32.033333333333303</v>
       </c>
-      <c r="AQ24" s="2">
+      <c r="AQ24" s="14">
         <v>13</v>
       </c>
-      <c r="AR24" s="2">
+      <c r="AR24" s="14">
         <v>32.769230769230802</v>
       </c>
-      <c r="AS24" s="2">
+      <c r="AS24" s="14">
         <v>34.2083333333333</v>
       </c>
-      <c r="AT24" s="9">
+      <c r="AT24" s="17">
         <v>41.142857142857103</v>
       </c>
-      <c r="AU24" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="AV24" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="AW24" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="AX24" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="AY24" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="AZ24" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BA24" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BB24" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BC24" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BD24" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BE24" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BF24" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BG24" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BH24" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BI24" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BJ24" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BK24" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BL24" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BM24" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BN24" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BO24" s="2">
+      <c r="AU24" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="AV24" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="AW24" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="AX24" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="AY24" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="AZ24" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BA24" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BB24" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BC24" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BD24" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BE24" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BF24" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BG24" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BH24" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BI24" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BJ24" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BK24" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BL24" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BM24" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BN24" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BO24" s="14">
         <v>4.7777777777777803</v>
       </c>
-      <c r="BP24" s="2">
+      <c r="BP24" s="14">
         <v>5.0833333333333304</v>
       </c>
-      <c r="BQ24" s="2">
+      <c r="BQ24" s="14">
         <v>2</v>
       </c>
-      <c r="BR24" s="2" t="s">
+      <c r="BR24" s="14" t="s">
         <v>124</v>
       </c>
-      <c r="BS24" s="2" t="s">
+      <c r="BS24" s="14" t="s">
         <v>125</v>
       </c>
-      <c r="BT24" s="2" t="s">
+      <c r="BT24" s="14" t="s">
         <v>126</v>
       </c>
-      <c r="BU24" s="2" t="s">
+      <c r="BU24" s="14" t="s">
         <v>127</v>
       </c>
-      <c r="BV24" s="2" t="s">
+      <c r="BV24" s="14" t="s">
         <v>118</v>
       </c>
-      <c r="BW24" s="2" t="s">
+      <c r="BW24" s="14" t="s">
         <v>92</v>
       </c>
-      <c r="BX24" s="2" t="s">
+      <c r="BX24" s="14" t="s">
         <v>104</v>
       </c>
-      <c r="BY24" s="13">
+      <c r="BY24" s="18">
         <v>45670</v>
       </c>
-      <c r="BZ24" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="CA24" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="CB24" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="CC24" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="CD24" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="CE24" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="CF24" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="CG24" s="2" t="s">
+      <c r="BZ24" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="CA24" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="CB24" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="CC24" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="CD24" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="CE24" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="CF24" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="CG24" s="14" t="s">
         <v>85</v>
       </c>
     </row>
@@ -7792,13 +7849,16 @@
         <v>186</v>
       </c>
       <c r="D25" t="s">
-        <v>200</v>
+        <v>199</v>
+      </c>
+      <c r="E25" t="s">
+        <v>208</v>
       </c>
       <c r="F25" s="1">
         <v>43317</v>
       </c>
-      <c r="G25" t="s">
-        <v>97</v>
+      <c r="G25" s="27" t="s">
+        <v>130</v>
       </c>
       <c r="H25" t="s">
         <v>122</v>
@@ -8035,508 +8095,514 @@
         <v>85</v>
       </c>
     </row>
-    <row r="26" spans="1:85" x14ac:dyDescent="0.3">
-      <c r="A26">
+    <row r="26" spans="1:85" s="19" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="19">
         <v>48998</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="19" t="s">
         <v>95</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C26" s="19" t="s">
         <v>187</v>
       </c>
-      <c r="D26" t="s">
-        <v>204</v>
-      </c>
-      <c r="F26" s="1">
+      <c r="D26" s="26" t="s">
+        <v>203</v>
+      </c>
+      <c r="E26" s="25" t="s">
+        <v>209</v>
+      </c>
+      <c r="F26" s="20">
         <v>43317</v>
       </c>
-      <c r="G26" s="4" t="s">
+      <c r="G26" s="21" t="s">
         <v>97</v>
       </c>
-      <c r="H26" t="s">
+      <c r="H26" s="19" t="s">
         <v>122</v>
       </c>
-      <c r="I26" t="s">
+      <c r="I26" s="19" t="s">
         <v>123</v>
       </c>
-      <c r="J26">
+      <c r="J26" s="19">
         <v>13998</v>
       </c>
-      <c r="K26">
+      <c r="K26" s="19">
         <v>3</v>
       </c>
-      <c r="L26">
+      <c r="L26" s="19">
         <v>43.602128999999998</v>
       </c>
-      <c r="M26" s="8">
+      <c r="M26" s="22">
         <v>-106.61529299999999</v>
       </c>
-      <c r="N26">
+      <c r="N26" s="19">
         <v>4</v>
       </c>
-      <c r="O26">
+      <c r="O26" s="19">
         <v>10</v>
       </c>
-      <c r="P26">
+      <c r="P26" s="19">
         <v>60</v>
       </c>
-      <c r="Q26">
+      <c r="Q26" s="19">
         <v>12</v>
       </c>
-      <c r="R26">
+      <c r="R26" s="19">
         <v>66</v>
       </c>
-      <c r="S26">
+      <c r="S26" s="19">
         <v>70.6666666666667</v>
       </c>
-      <c r="T26">
+      <c r="T26" s="19">
         <v>2</v>
       </c>
-      <c r="U26">
+      <c r="U26" s="19">
         <v>32</v>
       </c>
-      <c r="V26">
+      <c r="V26" s="19">
         <v>12.6666666666667</v>
       </c>
-      <c r="W26">
-        <v>0</v>
-      </c>
-      <c r="X26">
-        <v>0</v>
-      </c>
-      <c r="Y26">
+      <c r="W26" s="19">
+        <v>0</v>
+      </c>
+      <c r="X26" s="19">
+        <v>0</v>
+      </c>
+      <c r="Y26" s="19">
         <v>0.66666666666666696</v>
       </c>
-      <c r="Z26">
-        <v>0</v>
-      </c>
-      <c r="AA26">
+      <c r="Z26" s="19">
+        <v>0</v>
+      </c>
+      <c r="AA26" s="19">
         <v>14.6666666666667</v>
       </c>
-      <c r="AB26">
-        <v>0</v>
-      </c>
-      <c r="AC26">
-        <v>0</v>
-      </c>
-      <c r="AD26">
-        <v>0</v>
-      </c>
-      <c r="AE26">
+      <c r="AB26" s="19">
+        <v>0</v>
+      </c>
+      <c r="AC26" s="19">
+        <v>0</v>
+      </c>
+      <c r="AD26" s="19">
+        <v>0</v>
+      </c>
+      <c r="AE26" s="19">
         <v>14.6666666666667</v>
       </c>
-      <c r="AF26">
-        <v>0</v>
-      </c>
-      <c r="AG26">
-        <v>0</v>
-      </c>
-      <c r="AH26" s="8">
-        <v>0</v>
-      </c>
-      <c r="AI26">
+      <c r="AF26" s="19">
+        <v>0</v>
+      </c>
+      <c r="AG26" s="19">
+        <v>0</v>
+      </c>
+      <c r="AH26" s="22">
+        <v>0</v>
+      </c>
+      <c r="AI26" s="19">
         <v>1.67</v>
       </c>
-      <c r="AJ26">
+      <c r="AJ26" s="19">
         <v>1.27</v>
       </c>
-      <c r="AK26">
-        <v>0</v>
-      </c>
-      <c r="AL26">
-        <v>0</v>
-      </c>
-      <c r="AM26" s="8">
+      <c r="AK26" s="19">
+        <v>0</v>
+      </c>
+      <c r="AL26" s="19">
+        <v>0</v>
+      </c>
+      <c r="AM26" s="22">
         <v>2.94</v>
       </c>
-      <c r="AN26" s="4">
+      <c r="AN26" s="21">
         <v>36.727272727272698</v>
       </c>
-      <c r="AO26">
+      <c r="AO26" s="19">
         <v>34.1</v>
       </c>
-      <c r="AP26">
+      <c r="AP26" s="19">
         <v>34.1</v>
       </c>
-      <c r="AQ26" s="4">
+      <c r="AQ26" s="21">
         <v>21.4</v>
       </c>
-      <c r="AR26" s="4">
+      <c r="AR26" s="21">
         <v>35.409090909090899</v>
       </c>
-      <c r="AS26">
+      <c r="AS26" s="19">
         <v>39.529411764705898</v>
       </c>
-      <c r="AT26" s="8">
+      <c r="AT26" s="22">
         <v>46.9444444444444</v>
       </c>
-      <c r="AU26" t="s">
-        <v>85</v>
-      </c>
-      <c r="AV26" t="s">
-        <v>85</v>
-      </c>
-      <c r="AW26" t="s">
-        <v>85</v>
-      </c>
-      <c r="AX26" t="s">
-        <v>85</v>
-      </c>
-      <c r="AY26" t="s">
-        <v>85</v>
-      </c>
-      <c r="AZ26" t="s">
-        <v>85</v>
-      </c>
-      <c r="BA26" t="s">
-        <v>85</v>
-      </c>
-      <c r="BB26" t="s">
-        <v>85</v>
-      </c>
-      <c r="BC26" t="s">
-        <v>85</v>
-      </c>
-      <c r="BD26" t="s">
-        <v>85</v>
-      </c>
-      <c r="BE26" t="s">
-        <v>85</v>
-      </c>
-      <c r="BF26" t="s">
-        <v>85</v>
-      </c>
-      <c r="BG26" t="s">
-        <v>85</v>
-      </c>
-      <c r="BH26" t="s">
-        <v>85</v>
-      </c>
-      <c r="BI26" t="s">
-        <v>85</v>
-      </c>
-      <c r="BJ26" t="s">
-        <v>85</v>
-      </c>
-      <c r="BK26" t="s">
-        <v>85</v>
-      </c>
-      <c r="BL26" t="s">
-        <v>85</v>
-      </c>
-      <c r="BM26" t="s">
-        <v>85</v>
-      </c>
-      <c r="BN26" t="s">
-        <v>85</v>
-      </c>
-      <c r="BO26">
+      <c r="AU26" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="AV26" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="AW26" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="AX26" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="AY26" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="AZ26" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="BA26" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="BB26" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="BC26" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="BD26" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="BE26" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="BF26" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="BG26" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="BH26" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="BI26" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="BJ26" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="BK26" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="BL26" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="BM26" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="BN26" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="BO26" s="19">
         <v>5.7777777777777803</v>
       </c>
-      <c r="BP26">
+      <c r="BP26" s="19">
         <v>5.71428571428571</v>
       </c>
-      <c r="BQ26">
+      <c r="BQ26" s="19">
         <v>6</v>
       </c>
-      <c r="BR26" t="s">
+      <c r="BR26" s="19" t="s">
         <v>124</v>
       </c>
-      <c r="BS26" t="s">
+      <c r="BS26" s="19" t="s">
         <v>125</v>
       </c>
-      <c r="BT26" t="s">
+      <c r="BT26" s="19" t="s">
         <v>126</v>
       </c>
-      <c r="BU26" t="s">
+      <c r="BU26" s="19" t="s">
         <v>127</v>
       </c>
-      <c r="BV26" t="s">
+      <c r="BV26" s="19" t="s">
         <v>118</v>
       </c>
-      <c r="BW26" t="s">
+      <c r="BW26" s="19" t="s">
         <v>92</v>
       </c>
-      <c r="BX26" t="s">
+      <c r="BX26" s="19" t="s">
         <v>104</v>
       </c>
-      <c r="BY26" s="12">
+      <c r="BY26" s="23">
         <v>45670</v>
       </c>
-      <c r="BZ26" t="s">
-        <v>85</v>
-      </c>
-      <c r="CA26" t="s">
-        <v>85</v>
-      </c>
-      <c r="CB26" t="s">
-        <v>85</v>
-      </c>
-      <c r="CC26" t="s">
-        <v>85</v>
-      </c>
-      <c r="CD26" t="s">
-        <v>85</v>
-      </c>
-      <c r="CE26" t="s">
-        <v>85</v>
-      </c>
-      <c r="CF26" t="s">
-        <v>85</v>
-      </c>
-      <c r="CG26" t="s">
+      <c r="BZ26" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="CA26" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="CB26" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="CC26" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="CD26" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="CE26" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="CF26" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="CG26" s="19" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="27" spans="1:85" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="2">
+    <row r="27" spans="1:85" s="14" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="14">
         <v>48998</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="B27" s="14" t="s">
         <v>95</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="C27" s="14" t="s">
         <v>190</v>
       </c>
-      <c r="F27" s="3">
+      <c r="E27" s="14" t="s">
+        <v>209</v>
+      </c>
+      <c r="F27" s="15">
         <v>43317</v>
       </c>
-      <c r="G27" s="5" t="s">
+      <c r="G27" s="16" t="s">
         <v>130</v>
       </c>
-      <c r="H27" s="2" t="s">
+      <c r="H27" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="I27" s="2" t="s">
+      <c r="I27" s="14" t="s">
         <v>123</v>
       </c>
-      <c r="J27" s="2">
+      <c r="J27" s="14">
         <v>14887</v>
       </c>
-      <c r="K27" s="2">
+      <c r="K27" s="14">
         <v>3</v>
       </c>
-      <c r="L27" s="2">
+      <c r="L27" s="14">
         <v>43.602128999999998</v>
       </c>
-      <c r="M27" s="9">
+      <c r="M27" s="17">
         <v>-106.61529299999999</v>
       </c>
-      <c r="N27" s="2">
+      <c r="N27" s="14">
         <v>4</v>
       </c>
-      <c r="O27" s="2">
+      <c r="O27" s="14">
         <v>10</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="14">
         <v>60</v>
       </c>
-      <c r="Q27" s="2">
+      <c r="Q27" s="14">
         <v>12</v>
       </c>
-      <c r="R27" s="2">
+      <c r="R27" s="14">
         <v>66</v>
       </c>
-      <c r="S27" s="2">
+      <c r="S27" s="14">
         <v>70.6666666666667</v>
       </c>
-      <c r="T27" s="2">
+      <c r="T27" s="14">
         <v>2</v>
       </c>
-      <c r="U27" s="2">
+      <c r="U27" s="14">
         <v>32</v>
       </c>
-      <c r="V27" s="2">
+      <c r="V27" s="14">
         <v>12.6666666666667</v>
       </c>
-      <c r="W27" s="2">
-        <v>0</v>
-      </c>
-      <c r="X27" s="2">
-        <v>0</v>
-      </c>
-      <c r="Y27" s="2">
+      <c r="W27" s="14">
+        <v>0</v>
+      </c>
+      <c r="X27" s="14">
+        <v>0</v>
+      </c>
+      <c r="Y27" s="14">
         <v>0.66666666666666696</v>
       </c>
-      <c r="Z27" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA27" s="2">
+      <c r="Z27" s="14">
+        <v>0</v>
+      </c>
+      <c r="AA27" s="14">
         <v>14.6666666666667</v>
       </c>
-      <c r="AB27" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC27" s="2">
-        <v>0</v>
-      </c>
-      <c r="AD27" s="2">
-        <v>0</v>
-      </c>
-      <c r="AE27" s="2">
+      <c r="AB27" s="14">
+        <v>0</v>
+      </c>
+      <c r="AC27" s="14">
+        <v>0</v>
+      </c>
+      <c r="AD27" s="14">
+        <v>0</v>
+      </c>
+      <c r="AE27" s="14">
         <v>14.6666666666667</v>
       </c>
-      <c r="AF27" s="2">
-        <v>0</v>
-      </c>
-      <c r="AG27" s="2">
-        <v>0</v>
-      </c>
-      <c r="AH27" s="9">
-        <v>0</v>
-      </c>
-      <c r="AI27" s="2">
+      <c r="AF27" s="14">
+        <v>0</v>
+      </c>
+      <c r="AG27" s="14">
+        <v>0</v>
+      </c>
+      <c r="AH27" s="17">
+        <v>0</v>
+      </c>
+      <c r="AI27" s="14">
         <v>1.67</v>
       </c>
-      <c r="AJ27" s="2">
+      <c r="AJ27" s="14">
         <v>1.27</v>
       </c>
-      <c r="AK27" s="2">
-        <v>0</v>
-      </c>
-      <c r="AL27" s="2">
-        <v>0</v>
-      </c>
-      <c r="AM27" s="9">
+      <c r="AK27" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL27" s="14">
+        <v>0</v>
+      </c>
+      <c r="AM27" s="17">
         <v>2.94</v>
       </c>
-      <c r="AN27" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="AO27" s="2">
+      <c r="AN27" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="AO27" s="14">
         <v>34.1</v>
       </c>
-      <c r="AP27" s="2">
+      <c r="AP27" s="14">
         <v>34.1</v>
       </c>
-      <c r="AQ27" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="AR27" s="5">
+      <c r="AQ27" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="AR27" s="16">
         <v>39.529411764705898</v>
       </c>
-      <c r="AS27" s="2">
+      <c r="AS27" s="14">
         <v>39.529411764705898</v>
       </c>
-      <c r="AT27" s="9">
+      <c r="AT27" s="17">
         <v>46.9444444444444</v>
       </c>
-      <c r="AU27" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="AV27" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="AW27" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="AX27" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="AY27" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="AZ27" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BA27" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BB27" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BC27" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BD27" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BE27" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BF27" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BG27" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BH27" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BI27" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BJ27" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BK27" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BL27" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BM27" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BN27" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BO27" s="2">
+      <c r="AU27" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="AV27" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="AW27" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="AX27" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="AY27" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="AZ27" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BA27" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BB27" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BC27" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BD27" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BE27" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BF27" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BG27" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BH27" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BI27" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BJ27" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BK27" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BL27" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BM27" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BN27" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BO27" s="14">
         <v>5.7777777777777803</v>
       </c>
-      <c r="BP27" s="2">
+      <c r="BP27" s="14">
         <v>5.71428571428571</v>
       </c>
-      <c r="BQ27" s="2">
+      <c r="BQ27" s="14">
         <v>6</v>
       </c>
-      <c r="BR27" s="2" t="s">
+      <c r="BR27" s="14" t="s">
         <v>124</v>
       </c>
-      <c r="BS27" s="2" t="s">
+      <c r="BS27" s="14" t="s">
         <v>125</v>
       </c>
-      <c r="BT27" s="2" t="s">
+      <c r="BT27" s="14" t="s">
         <v>126</v>
       </c>
-      <c r="BU27" s="2" t="s">
+      <c r="BU27" s="14" t="s">
         <v>127</v>
       </c>
-      <c r="BV27" s="2" t="s">
+      <c r="BV27" s="14" t="s">
         <v>118</v>
       </c>
-      <c r="BW27" s="2" t="s">
+      <c r="BW27" s="14" t="s">
         <v>92</v>
       </c>
-      <c r="BX27" s="2" t="s">
+      <c r="BX27" s="14" t="s">
         <v>104</v>
       </c>
-      <c r="BY27" s="13">
+      <c r="BY27" s="18">
         <v>45670</v>
       </c>
-      <c r="BZ27" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="CA27" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="CB27" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="CC27" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="CD27" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="CE27" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="CF27" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="CG27" s="2" t="s">
+      <c r="BZ27" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="CA27" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="CB27" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="CC27" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="CD27" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="CE27" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="CF27" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="CG27" s="14" t="s">
         <v>85</v>
       </c>
     </row>
@@ -9056,16 +9122,16 @@
         <v>140</v>
       </c>
       <c r="D30" t="s">
-        <v>199</v>
+        <v>210</v>
       </c>
       <c r="E30" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F30" s="1">
         <v>43261</v>
       </c>
-      <c r="G30" s="4" t="s">
-        <v>97</v>
+      <c r="G30" s="24" t="s">
+        <v>142</v>
       </c>
       <c r="H30" t="s">
         <v>122</v>
@@ -9312,6 +9378,9 @@
       <c r="C31" s="14" t="s">
         <v>141</v>
       </c>
+      <c r="E31" s="14" t="s">
+        <v>209</v>
+      </c>
       <c r="F31" s="15">
         <v>43261</v>
       </c>
@@ -9564,7 +9633,7 @@
         <v>112</v>
       </c>
       <c r="D32" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F32" s="1">
         <v>42927</v>
@@ -10068,11 +10137,17 @@
       <c r="C34" t="s">
         <v>157</v>
       </c>
+      <c r="D34" t="s">
+        <v>210</v>
+      </c>
+      <c r="E34" t="s">
+        <v>208</v>
+      </c>
       <c r="F34" s="1">
         <v>43271</v>
       </c>
-      <c r="G34" t="s">
-        <v>97</v>
+      <c r="G34" s="24" t="s">
+        <v>130</v>
       </c>
       <c r="H34" t="s">
         <v>122</v>
@@ -10284,279 +10359,282 @@
       <c r="BY34" s="12">
         <v>45670</v>
       </c>
-      <c r="BZ34">
-        <v>0</v>
-      </c>
-      <c r="CA34">
-        <v>0</v>
-      </c>
-      <c r="CB34">
-        <v>0</v>
-      </c>
-      <c r="CC34">
-        <v>0</v>
-      </c>
-      <c r="CD34">
+      <c r="BZ34" s="4">
+        <v>0</v>
+      </c>
+      <c r="CA34" s="4">
+        <v>0</v>
+      </c>
+      <c r="CB34" s="4">
+        <v>0</v>
+      </c>
+      <c r="CC34" s="4">
+        <v>0</v>
+      </c>
+      <c r="CD34" s="4">
         <v>307</v>
       </c>
-      <c r="CE34">
+      <c r="CE34" s="4">
         <v>11</v>
       </c>
-      <c r="CF34">
-        <v>0</v>
-      </c>
-      <c r="CG34">
+      <c r="CF34" s="4">
+        <v>0</v>
+      </c>
+      <c r="CG34" s="4">
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:85" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="2">
+    <row r="35" spans="1:85" s="14" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="14">
         <v>49740</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="B35" s="14" t="s">
         <v>95</v>
       </c>
-      <c r="C35" s="2" t="s">
+      <c r="C35" s="14" t="s">
         <v>158</v>
       </c>
-      <c r="F35" s="3">
+      <c r="E35" s="14" t="s">
+        <v>209</v>
+      </c>
+      <c r="F35" s="15">
         <v>43271</v>
       </c>
-      <c r="G35" s="2" t="s">
+      <c r="G35" s="16" t="s">
         <v>130</v>
       </c>
-      <c r="H35" s="2" t="s">
+      <c r="H35" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="I35" s="2" t="s">
+      <c r="I35" s="14" t="s">
         <v>123</v>
       </c>
-      <c r="J35" s="2">
+      <c r="J35" s="14">
         <v>13072</v>
       </c>
-      <c r="K35" s="2">
+      <c r="K35" s="14">
         <v>2</v>
       </c>
-      <c r="L35" s="2">
+      <c r="L35" s="14">
         <v>43.771549999999998</v>
       </c>
-      <c r="M35" s="9">
+      <c r="M35" s="17">
         <v>-106.78945</v>
       </c>
-      <c r="N35" s="2">
+      <c r="N35" s="14">
         <v>0.66666666666666696</v>
       </c>
-      <c r="O35" s="2">
+      <c r="O35" s="14">
         <v>3.3333333333333299</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="14">
         <v>14.6666666666667</v>
       </c>
-      <c r="Q35" s="2">
+      <c r="Q35" s="14">
         <v>6</v>
       </c>
-      <c r="R35" s="2">
+      <c r="R35" s="14">
         <v>16.6666666666667</v>
       </c>
-      <c r="S35" s="2">
+      <c r="S35" s="14">
         <v>88.6666666666667</v>
       </c>
-      <c r="T35" s="2">
+      <c r="T35" s="14">
         <v>2.6666666666666701</v>
       </c>
-      <c r="U35" s="2">
+      <c r="U35" s="14">
         <v>84.6666666666667</v>
       </c>
-      <c r="V35" s="2">
-        <v>0</v>
-      </c>
-      <c r="W35" s="2">
-        <v>0</v>
-      </c>
-      <c r="X35" s="2">
-        <v>0</v>
-      </c>
-      <c r="Y35" s="2">
-        <v>0</v>
-      </c>
-      <c r="Z35" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA35" s="2">
+      <c r="V35" s="14">
+        <v>0</v>
+      </c>
+      <c r="W35" s="14">
+        <v>0</v>
+      </c>
+      <c r="X35" s="14">
+        <v>0</v>
+      </c>
+      <c r="Y35" s="14">
+        <v>0</v>
+      </c>
+      <c r="Z35" s="14">
+        <v>0</v>
+      </c>
+      <c r="AA35" s="14">
         <v>9.3333333333333304</v>
       </c>
-      <c r="AB35" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC35" s="2">
-        <v>0</v>
-      </c>
-      <c r="AD35" s="2">
-        <v>0</v>
-      </c>
-      <c r="AE35" s="2">
+      <c r="AB35" s="14">
+        <v>0</v>
+      </c>
+      <c r="AC35" s="14">
+        <v>0</v>
+      </c>
+      <c r="AD35" s="14">
+        <v>0</v>
+      </c>
+      <c r="AE35" s="14">
         <v>9.3333333333333304</v>
       </c>
-      <c r="AF35" s="2">
-        <v>0</v>
-      </c>
-      <c r="AG35" s="2">
-        <v>0</v>
-      </c>
-      <c r="AH35" s="9">
-        <v>0</v>
-      </c>
-      <c r="AI35" s="2">
+      <c r="AF35" s="14">
+        <v>0</v>
+      </c>
+      <c r="AG35" s="14">
+        <v>0</v>
+      </c>
+      <c r="AH35" s="17">
+        <v>0</v>
+      </c>
+      <c r="AI35" s="14">
         <v>1.88</v>
       </c>
-      <c r="AJ35" s="2">
-        <v>0</v>
-      </c>
-      <c r="AK35" s="2">
-        <v>0</v>
-      </c>
-      <c r="AL35" s="2">
-        <v>0</v>
-      </c>
-      <c r="AM35" s="9">
+      <c r="AJ35" s="14">
+        <v>0</v>
+      </c>
+      <c r="AK35" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL35" s="14">
+        <v>0</v>
+      </c>
+      <c r="AM35" s="17">
         <v>1.88</v>
       </c>
-      <c r="AN35" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="AO35" s="2">
+      <c r="AN35" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="AO35" s="14">
         <v>30.866666666666699</v>
       </c>
-      <c r="AP35" s="2">
+      <c r="AP35" s="14">
         <v>30.866666666666699</v>
       </c>
-      <c r="AQ35" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="AR35" s="2">
+      <c r="AQ35" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="AR35" s="14">
         <v>31.296296296296301</v>
       </c>
-      <c r="AS35" s="2">
+      <c r="AS35" s="14">
         <v>31.296296296296301</v>
       </c>
-      <c r="AT35" s="9">
+      <c r="AT35" s="17">
         <v>15.818181818181801</v>
       </c>
-      <c r="AU35" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="AV35" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="AW35" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="AX35" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="AY35" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="AZ35" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BA35" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BB35" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BC35" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BD35" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BE35" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BF35" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BG35" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BH35" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BI35" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BJ35" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BK35" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BL35" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BM35" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BN35" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="BO35" s="2">
+      <c r="AU35" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="AV35" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="AW35" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="AX35" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="AY35" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="AZ35" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BA35" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BB35" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BC35" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BD35" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BE35" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BF35" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BG35" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BH35" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BI35" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BJ35" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BK35" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BL35" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BM35" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BN35" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="BO35" s="14">
         <v>4.1666666666666696</v>
       </c>
-      <c r="BP35" s="2">
+      <c r="BP35" s="14">
         <v>4.5</v>
       </c>
-      <c r="BQ35" s="2">
+      <c r="BQ35" s="14">
         <v>3.5</v>
       </c>
-      <c r="BR35" s="2" t="s">
+      <c r="BR35" s="14" t="s">
         <v>99</v>
       </c>
-      <c r="BS35" s="2" t="s">
+      <c r="BS35" s="14" t="s">
         <v>100</v>
       </c>
-      <c r="BT35" s="2" t="s">
+      <c r="BT35" s="14" t="s">
         <v>131</v>
       </c>
-      <c r="BU35" s="2" t="s">
+      <c r="BU35" s="14" t="s">
         <v>132</v>
       </c>
-      <c r="BV35" s="2" t="s">
+      <c r="BV35" s="14" t="s">
         <v>118</v>
       </c>
-      <c r="BW35" s="2" t="s">
+      <c r="BW35" s="14" t="s">
         <v>92</v>
       </c>
-      <c r="BX35" s="2" t="s">
+      <c r="BX35" s="14" t="s">
         <v>104</v>
       </c>
-      <c r="BY35" s="13">
+      <c r="BY35" s="18">
         <v>45670</v>
       </c>
-      <c r="BZ35" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="CA35" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="CB35" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="CC35" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="CD35" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="CE35" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="CF35" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="CG35" s="2" t="s">
+      <c r="BZ35" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="CA35" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="CB35" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="CC35" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="CD35" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="CE35" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="CF35" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="CG35" s="16" t="s">
         <v>85</v>
       </c>
     </row>
@@ -10571,16 +10649,16 @@
         <v>134</v>
       </c>
       <c r="D36" t="s">
-        <v>199</v>
+        <v>210</v>
       </c>
       <c r="E36" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F36" s="1">
         <v>43255</v>
       </c>
-      <c r="G36" s="4" t="s">
-        <v>97</v>
+      <c r="G36" s="24" t="s">
+        <v>137</v>
       </c>
       <c r="H36" t="s">
         <v>122</v>
@@ -10828,7 +10906,7 @@
         <v>136</v>
       </c>
       <c r="E37" s="14" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F37" s="15">
         <v>43255</v>
@@ -11082,16 +11160,16 @@
         <v>148</v>
       </c>
       <c r="D38" t="s">
-        <v>199</v>
+        <v>210</v>
       </c>
       <c r="E38" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F38" s="1">
         <v>43269</v>
       </c>
-      <c r="G38" s="4" t="s">
-        <v>97</v>
+      <c r="G38" s="24" t="s">
+        <v>130</v>
       </c>
       <c r="H38" t="s">
         <v>122</v>
@@ -11339,7 +11417,7 @@
         <v>149</v>
       </c>
       <c r="E39" s="14" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F39" s="15">
         <v>43269</v>
@@ -11593,16 +11671,16 @@
         <v>143</v>
       </c>
       <c r="D40" t="s">
-        <v>199</v>
+        <v>210</v>
       </c>
       <c r="E40" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F40" s="1">
         <v>43263</v>
       </c>
-      <c r="G40" s="4" t="s">
-        <v>97</v>
+      <c r="G40" s="24" t="s">
+        <v>145</v>
       </c>
       <c r="H40" t="s">
         <v>122</v>
@@ -11850,7 +11928,7 @@
         <v>144</v>
       </c>
       <c r="E41" s="14" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F41" s="15">
         <v>43263</v>
@@ -12104,16 +12182,16 @@
         <v>146</v>
       </c>
       <c r="D42" t="s">
-        <v>199</v>
+        <v>210</v>
       </c>
       <c r="E42" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F42" s="1">
         <v>43263</v>
       </c>
-      <c r="G42" s="4" t="s">
-        <v>97</v>
+      <c r="G42" s="24" t="s">
+        <v>137</v>
       </c>
       <c r="H42" t="s">
         <v>122</v>
@@ -12361,7 +12439,7 @@
         <v>147</v>
       </c>
       <c r="E43" s="14" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F43" s="15">
         <v>43263</v>
@@ -12615,10 +12693,10 @@
         <v>181</v>
       </c>
       <c r="D44" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E44" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F44" s="1">
         <v>43305</v>
@@ -12872,7 +12950,7 @@
         <v>182</v>
       </c>
       <c r="E45" s="14" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F45" s="15">
         <v>43305</v>
@@ -13126,10 +13204,10 @@
         <v>178</v>
       </c>
       <c r="D46" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E46" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F46" s="1">
         <v>43305</v>
@@ -13383,7 +13461,7 @@
         <v>180</v>
       </c>
       <c r="E47" s="14" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F47" s="15">
         <v>43305</v>
@@ -13637,16 +13715,16 @@
         <v>138</v>
       </c>
       <c r="D48" t="s">
-        <v>199</v>
+        <v>210</v>
       </c>
       <c r="E48" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F48" s="1">
         <v>43265</v>
       </c>
-      <c r="G48" s="4" t="s">
-        <v>97</v>
+      <c r="G48" s="24" t="s">
+        <v>130</v>
       </c>
       <c r="H48" t="s">
         <v>122</v>
@@ -13894,7 +13972,7 @@
         <v>139</v>
       </c>
       <c r="E49" s="14" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F49" s="15">
         <v>43265</v>
@@ -14148,10 +14226,10 @@
         <v>183</v>
       </c>
       <c r="D50" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E50" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F50" s="1">
         <v>43306</v>
@@ -14405,7 +14483,7 @@
         <v>185</v>
       </c>
       <c r="E51" s="14" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F51" s="15">
         <v>43306</v>
@@ -14659,10 +14737,10 @@
         <v>174</v>
       </c>
       <c r="D52" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E52" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F52" s="1">
         <v>43304</v>
@@ -14916,7 +14994,7 @@
         <v>177</v>
       </c>
       <c r="E53" s="14" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F53" s="15">
         <v>43304</v>
@@ -15170,13 +15248,13 @@
         <v>170</v>
       </c>
       <c r="D54" t="s">
-        <v>199</v>
+        <v>210</v>
       </c>
       <c r="F54" s="1">
         <v>43277</v>
       </c>
-      <c r="G54" s="4" t="s">
-        <v>97</v>
+      <c r="G54" s="24" t="s">
+        <v>121</v>
       </c>
       <c r="H54" t="s">
         <v>122</v>
@@ -15424,7 +15502,7 @@
         <v>171</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="F55" s="3">
         <v>43277</v>
@@ -15678,16 +15756,16 @@
         <v>161</v>
       </c>
       <c r="D56" t="s">
-        <v>199</v>
+        <v>210</v>
       </c>
       <c r="E56" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F56" s="1">
         <v>43276</v>
       </c>
-      <c r="G56" s="4" t="s">
-        <v>97</v>
+      <c r="G56" s="24" t="s">
+        <v>163</v>
       </c>
       <c r="H56" t="s">
         <v>122</v>
@@ -15935,7 +16013,7 @@
         <v>162</v>
       </c>
       <c r="E57" s="14" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F57" s="15">
         <v>43276</v>
@@ -16189,7 +16267,10 @@
         <v>172</v>
       </c>
       <c r="D58" t="s">
-        <v>199</v>
+        <v>210</v>
+      </c>
+      <c r="E58" t="s">
+        <v>208</v>
       </c>
       <c r="F58" s="1">
         <v>43285</v>
@@ -16443,7 +16524,10 @@
         <v>173</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
+      </c>
+      <c r="E59" s="2" t="s">
+        <v>209</v>
       </c>
       <c r="F59" s="3">
         <v>43285</v>
@@ -16697,13 +16781,13 @@
         <v>167</v>
       </c>
       <c r="D60" t="s">
-        <v>199</v>
+        <v>210</v>
       </c>
       <c r="F60" s="1">
         <v>43277</v>
       </c>
-      <c r="G60" s="4" t="s">
-        <v>97</v>
+      <c r="G60" s="24" t="s">
+        <v>137</v>
       </c>
       <c r="H60" t="s">
         <v>122</v>
@@ -16951,7 +17035,7 @@
         <v>169</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F61" s="3">
         <v>43277</v>
@@ -17205,16 +17289,16 @@
         <v>164</v>
       </c>
       <c r="D62" t="s">
-        <v>199</v>
+        <v>210</v>
       </c>
       <c r="E62" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F62" s="1">
         <v>43276</v>
       </c>
-      <c r="G62" s="4" t="s">
-        <v>97</v>
+      <c r="G62" s="24" t="s">
+        <v>163</v>
       </c>
       <c r="H62" t="s">
         <v>122</v>
@@ -17462,7 +17546,7 @@
         <v>166</v>
       </c>
       <c r="E63" s="19" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F63" s="20">
         <v>43276</v>

</xml_diff>